<commit_message>
Added eqns for unknown conifer
</commit_message>
<xml_diff>
--- a/WoodyBiomassEqns.xlsx
+++ b/WoodyBiomassEqns.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pointblue-my.sharepoint.com/personal/leash_pointblue_org/Documents/Documents/AgC/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pointblue-my.sharepoint.com/personal/acook_pointblue_org/Documents/Documents/AgC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3C3A27CC-853E-4196-8A2D-5967ABB1553A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="8_{3C3A27CC-853E-4196-8A2D-5967ABB1553A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B251DDD-FE5B-4446-8948-6110DCE04576}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BE8BCD95-B122-4CEB-8FDD-710E9DA2E420}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BE8BCD95-B122-4CEB-8FDD-710E9DA2E420}"/>
   </bookViews>
   <sheets>
     <sheet name="Species_database" sheetId="8" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="193">
   <si>
     <t>genus</t>
   </si>
@@ -608,6 +608,15 @@
   </si>
   <si>
     <t>Unknown</t>
+  </si>
+  <si>
+    <t>Unknown conifer</t>
+  </si>
+  <si>
+    <t>Conifer</t>
+  </si>
+  <si>
+    <t>289/299</t>
   </si>
 </sst>
 </file>
@@ -2522,18 +2531,69 @@
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="H26" s="5"/>
-      <c r="I26" s="5"/>
-      <c r="J26" s="5"/>
-      <c r="K26" s="5"/>
-      <c r="M26" s="5"/>
-      <c r="N26" s="5"/>
-      <c r="O26" s="5"/>
-      <c r="P26" s="5"/>
-      <c r="R26" s="5"/>
-      <c r="S26" s="5"/>
-      <c r="T26" s="5"/>
-      <c r="U26" s="5"/>
+      <c r="A26" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F26">
+        <v>25.58</v>
+      </c>
+      <c r="G26" s="4">
+        <v>17</v>
+      </c>
+      <c r="H26" s="5">
+        <v>17</v>
+      </c>
+      <c r="I26" s="5">
+        <v>17</v>
+      </c>
+      <c r="J26" s="5">
+        <v>17</v>
+      </c>
+      <c r="K26" s="5">
+        <v>17</v>
+      </c>
+      <c r="L26" s="4">
+        <v>21</v>
+      </c>
+      <c r="M26" s="5">
+        <v>21</v>
+      </c>
+      <c r="N26" s="5">
+        <v>21</v>
+      </c>
+      <c r="O26" s="5">
+        <v>21</v>
+      </c>
+      <c r="P26" s="5">
+        <v>21</v>
+      </c>
+      <c r="Q26" s="4">
+        <v>24</v>
+      </c>
+      <c r="R26" s="5">
+        <v>24</v>
+      </c>
+      <c r="S26" s="5">
+        <v>24</v>
+      </c>
+      <c r="T26" s="5">
+        <v>24</v>
+      </c>
+      <c r="U26" s="5">
+        <v>24</v>
+      </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.35">
       <c r="H27" s="5"/>
@@ -4916,26 +4976,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="517e5903-1e8c-4d3d-8c4e-1f79952d16c1" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="8f76b250-a6d5-4c52-a304-c508ae7b4989">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B6C9CDEE2418C348959EA02F5D8F9961" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bd29e3ab8a1c22d4e4b1d57fe712065d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8f76b250-a6d5-4c52-a304-c508ae7b4989" xmlns:ns3="517e5903-1e8c-4d3d-8c4e-1f79952d16c1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1fa30353a3bab6554c5e779678dd4025" ns2:_="" ns3:_="">
     <xsd:import namespace="8f76b250-a6d5-4c52-a304-c508ae7b4989"/>
@@ -5170,26 +5210,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD233B28-259D-43DA-A5BD-0382CE33D615}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="517e5903-1e8c-4d3d-8c4e-1f79952d16c1"/>
-    <ds:schemaRef ds:uri="8f76b250-a6d5-4c52-a304-c508ae7b4989"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{337F3735-3D4E-4CCF-A8A8-E79896DB19B5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="517e5903-1e8c-4d3d-8c4e-1f79952d16c1" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="8f76b250-a6d5-4c52-a304-c508ae7b4989">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9DB875A-592E-4F1F-8784-348A5BBED7BD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5206,4 +5247,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{337F3735-3D4E-4CCF-A8A8-E79896DB19B5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD233B28-259D-43DA-A5BD-0382CE33D615}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="517e5903-1e8c-4d3d-8c4e-1f79952d16c1"/>
+    <ds:schemaRef ds:uri="8f76b250-a6d5-4c52-a304-c508ae7b4989"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>